<commit_message>
feature/fsel-3838: Update Code Manager Report Learning Progress, Learning Result , Student Assiduity
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoPlacmentTest.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoPlacmentTest.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PhanPhuc\Fsel\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ExcelTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2547401-0051-4CA3-899C-BB997E90158D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{316E1724-6FA7-47E6-AF46-1F428B0E0294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0455E090-DA9A-40C9-A1B2-4E43F6F76E19}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0455E090-DA9A-40C9-A1B2-4E43F6F76E19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="179021" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="31">
   <si>
     <t>BÁO CÁO KẾT QUẢ BÀI KIỂM TRA ĐẦU VÀO</t>
   </si>
@@ -33,6 +33,9 @@
     <t>Trường</t>
   </si>
   <si>
+    <t>[SchoolName]</t>
+  </si>
+  <si>
     <t>Tổng số học sinh</t>
   </si>
   <si>
@@ -66,13 +69,37 @@
     <t>Khóa học lựa chọn</t>
   </si>
   <si>
+    <t>Trình độ hiện trại</t>
+  </si>
+  <si>
     <t>Trạng thái</t>
   </si>
   <si>
     <t>Ngày kết thúc</t>
   </si>
   <si>
-    <t>{0}</t>
+    <t>Ngày: {0}</t>
+  </si>
+  <si>
+    <t>Đến ngày: {0}</t>
+  </si>
+  <si>
+    <t>Từ ngày: {0}</t>
+  </si>
+  <si>
+    <t>Khóa học: {0}</t>
+  </si>
+  <si>
+    <t>Trình độ: {0}</t>
+  </si>
+  <si>
+    <t>Lớp: {0}</t>
+  </si>
+  <si>
+    <t>Khối: {0}</t>
+  </si>
+  <si>
+    <t>Trạng thái: {0}</t>
   </si>
   <si>
     <t>A1: {0}</t>
@@ -91,24 +118,6 @@
   </si>
   <si>
     <t>C1: {0}</t>
-  </si>
-  <si>
-    <t>Ngày: {0}</t>
-  </si>
-  <si>
-    <t>Đến ngày: {0}</t>
-  </si>
-  <si>
-    <t>Từ ngày: {0}</t>
-  </si>
-  <si>
-    <t>Khối: {0}</t>
-  </si>
-  <si>
-    <t>Trạng thái: {0}</t>
-  </si>
-  <si>
-    <t>Trình độ hiện tại</t>
   </si>
 </sst>
 </file>
@@ -124,20 +133,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="20"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -145,17 +140,34 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="20"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="5">
@@ -164,12 +176,6 @@
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDBDBDB"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -183,8 +189,14 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD0CECE"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -194,11 +206,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
       </left>
       <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -207,14 +232,25 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
@@ -222,13 +258,22 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -237,14 +282,12 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -258,39 +301,72 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -609,203 +685,218 @@
   <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="38.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.75" customWidth="1"/>
+    <col min="6" max="6" width="24.375" customWidth="1"/>
     <col min="7" max="7" width="18.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.25" customWidth="1"/>
-    <col min="9" max="9" width="17.375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.125" customWidth="1"/>
+    <col min="9" max="9" width="35.125" customWidth="1"/>
+    <col min="10" max="10" width="29.125" customWidth="1"/>
+    <col min="11" max="11" width="40.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="12" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A2" s="2"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="3" t="s">
+    <row r="2" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="13"/>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
+      <c r="H3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A3" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="3" t="s">
+    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15">
+        <v>150</v>
+      </c>
+      <c r="E4" s="15"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="8"/>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15">
+        <v>100</v>
+      </c>
+      <c r="E5" s="15"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="8"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15">
+        <v>80</v>
+      </c>
+      <c r="E6" s="15"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="8"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A4" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="7"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A5" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="7"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A7" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
+      <c r="F7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7" s="10"/>
+      <c r="K7" s="11"/>
     </row>
     <row r="8" spans="1:11" ht="30" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="10" t="s">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="C8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="D8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="10" t="s">
+      <c r="F8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="G8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I8" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="10" t="s">
+      <c r="H8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="I8" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
+      <c r="A9" s="1"/>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
+  <mergeCells count="10">
+    <mergeCell ref="K1:K2"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="A1:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feature/fsel-6191: Update Code Export File Report
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoPlacmentTest.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ManagerReports/BaoCaoPlacmentTest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ManagerReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753FAE5C-EEFA-4C3B-B6BE-15998088A49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E6AC0CC-4569-440B-8FA7-6D0D2197E04B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0455E090-DA9A-40C9-A1B2-4E43F6F76E19}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>BÁO CÁO KẾT QUẢ BÀI KIỂM TRA ĐẦU VÀO</t>
   </si>
@@ -121,13 +121,16 @@
   </si>
   <si>
     <t>Trạng thái: {0}</t>
+  </si>
+  <si>
+    <t>0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,41 +139,34 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
+      <b/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
     </font>
     <font>
-      <b/>
-      <sz val="20"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <scheme val="major"/>
     </font>
   </fonts>
   <fills count="5">
@@ -306,62 +302,62 @@
   </cellStyleXfs>
   <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -677,205 +673,206 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8FF2C25-AFD5-447B-8DDE-AACBEAB174E4}">
   <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="29" customWidth="1"/>
-    <col min="3" max="3" width="18.5" customWidth="1"/>
-    <col min="4" max="4" width="19.25" customWidth="1"/>
-    <col min="5" max="5" width="17.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.375" customWidth="1"/>
-    <col min="7" max="7" width="18.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33.125" customWidth="1"/>
-    <col min="9" max="9" width="35.125" customWidth="1"/>
-    <col min="10" max="10" width="29.125" customWidth="1"/>
-    <col min="11" max="11" width="40.75" customWidth="1"/>
+    <col min="1" max="2" width="29" style="20" customWidth="1"/>
+    <col min="3" max="3" width="18.5" style="20" customWidth="1"/>
+    <col min="4" max="4" width="19.25" style="20" customWidth="1"/>
+    <col min="5" max="5" width="17.375" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.375" style="20" customWidth="1"/>
+    <col min="7" max="7" width="18.125" style="20" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.125" style="20" customWidth="1"/>
+    <col min="9" max="9" width="35.125" style="20" customWidth="1"/>
+    <col min="10" max="10" width="29.125" style="20" customWidth="1"/>
+    <col min="11" max="11" width="40.75" style="20" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="20"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="13" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="14"/>
+    <row r="2" spans="1:11" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="21"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="4" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="12" t="s">
+      <c r="E3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="K3" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="12">
-        <v>150</v>
-      </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="20"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="10"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="12"/>
+      <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="12">
-        <v>100</v>
-      </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="8"/>
-      <c r="K5" s="20"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="9"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="12">
-        <v>80</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="8"/>
-      <c r="K6" s="20"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="22"/>
-      <c r="D7" s="9" t="s">
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H7" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="11"/>
-      <c r="K7" s="20"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="9"/>
     </row>
-    <row r="8" spans="1:11" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="K8" s="23" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="J9" s="24"/>
+      <c r="K9" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>